<commit_message>
update supply slack implementation
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB5F6F3-D612-40F9-BF71-3716FB7E0E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D20B0F-9124-42F1-8BC3-38155DD48764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -1601,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>81</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1634,7 +1634,7 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>81</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
bug fix node preparation
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D20B0F-9124-42F1-8BC3-38155DD48764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C31F195-39CA-4D76-8A32-E81E4AE03078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
@@ -1711,7 +1711,7 @@
         <v>19</v>
       </c>
       <c r="C13">
-        <v>-5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
test undirected flow example
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C31F195-39CA-4D76-8A32-E81E4AE03078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB356B6F-766F-4F18-A8F2-97277EE6B7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
bidirectional flow script testing
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data_update.xlsx
+++ b/01_data/01_input_data/02_processed/Data_update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB356B6F-766F-4F18-A8F2-97277EE6B7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3607DD-2064-45FC-B483-AD4F3C3E5AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
@@ -1601,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>60</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1634,7 +1634,7 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>